<commit_message>
Add manual test cases
</commit_message>
<xml_diff>
--- a/input/youtube-tests.xlsx
+++ b/input/youtube-tests.xlsx
@@ -1,17 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <workbookPr filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="600" windowWidth="19815" windowHeight="7110"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="ManualTestCases" state="visible" r:id="rId4"/>
+    <sheet name="ManualTestCases" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="176">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -536,22 +539,27 @@
   </si>
   <si>
     <t>The browser returns to the video</t>
+  </si>
+  <si>
+    <t>Enter "playwright automation tutorial in tamil" in the search box</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -915,9 +923,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E219"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -926,7 +934,7 @@
     <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -943,7 +951,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -960,7 +968,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -977,7 +985,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -994,7 +1002,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1011,7 +1019,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1028,7 +1036,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1045,7 +1053,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1062,7 +1070,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1079,7 +1087,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1096,7 +1104,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1113,7 +1121,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1130,7 +1138,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1147,7 +1155,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1164,7 +1172,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1181,7 +1189,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1198,7 +1206,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1215,7 +1223,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1232,7 +1240,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -1249,7 +1257,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1266,7 +1274,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -1283,7 +1291,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -1300,7 +1308,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1317,7 +1325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -1334,7 +1342,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
         <v>36</v>
       </c>
@@ -1351,7 +1359,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1368,7 +1376,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -1385,7 +1393,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -1402,7 +1410,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -1419,7 +1427,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -1436,7 +1444,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -1453,7 +1461,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -1470,7 +1478,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -1487,7 +1495,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -1504,7 +1512,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -1521,7 +1529,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -1538,7 +1546,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -1555,7 +1563,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -1572,7 +1580,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
         <v>48</v>
       </c>
@@ -1589,7 +1597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -1606,7 +1614,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5">
       <c r="A41" t="s">
         <v>48</v>
       </c>
@@ -1623,7 +1631,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -1640,7 +1648,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -1657,7 +1665,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -1674,7 +1682,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5">
       <c r="A45" t="s">
         <v>52</v>
       </c>
@@ -1691,7 +1699,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -1708,7 +1716,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1725,7 +1733,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -1742,7 +1750,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5">
       <c r="A49" t="s">
         <v>52</v>
       </c>
@@ -1759,7 +1767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5">
       <c r="A50" t="s">
         <v>52</v>
       </c>
@@ -1776,7 +1784,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5">
       <c r="A51" t="s">
         <v>52</v>
       </c>
@@ -1793,7 +1801,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5">
       <c r="A52" t="s">
         <v>52</v>
       </c>
@@ -1810,7 +1818,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -1827,7 +1835,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -1844,7 +1852,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -1861,7 +1869,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5">
       <c r="A56" t="s">
         <v>58</v>
       </c>
@@ -1878,7 +1886,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5">
       <c r="A57" t="s">
         <v>58</v>
       </c>
@@ -1895,7 +1903,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5">
       <c r="A58" t="s">
         <v>58</v>
       </c>
@@ -1912,7 +1920,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5">
       <c r="A59" t="s">
         <v>63</v>
       </c>
@@ -1929,7 +1937,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5">
       <c r="A60" t="s">
         <v>63</v>
       </c>
@@ -1946,7 +1954,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5">
       <c r="A61" t="s">
         <v>63</v>
       </c>
@@ -1963,7 +1971,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -1980,7 +1988,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5">
       <c r="A63" t="s">
         <v>63</v>
       </c>
@@ -1997,7 +2005,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -2014,7 +2022,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -2031,7 +2039,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5">
       <c r="A66" t="s">
         <v>63</v>
       </c>
@@ -2048,7 +2056,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5">
       <c r="A67" t="s">
         <v>66</v>
       </c>
@@ -2065,7 +2073,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5">
       <c r="A68" t="s">
         <v>66</v>
       </c>
@@ -2082,7 +2090,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5">
       <c r="A69" t="s">
         <v>66</v>
       </c>
@@ -2099,7 +2107,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5">
       <c r="A70" t="s">
         <v>66</v>
       </c>
@@ -2116,7 +2124,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -2133,7 +2141,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5">
       <c r="A72" t="s">
         <v>70</v>
       </c>
@@ -2150,7 +2158,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5">
       <c r="A73" t="s">
         <v>70</v>
       </c>
@@ -2167,7 +2175,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5">
       <c r="A74" t="s">
         <v>70</v>
       </c>
@@ -2184,7 +2192,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5">
       <c r="A75" t="s">
         <v>70</v>
       </c>
@@ -2201,7 +2209,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5">
       <c r="A76" t="s">
         <v>70</v>
       </c>
@@ -2218,7 +2226,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5">
       <c r="A77" t="s">
         <v>70</v>
       </c>
@@ -2235,7 +2243,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5">
       <c r="A78" t="s">
         <v>70</v>
       </c>
@@ -2252,7 +2260,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5">
       <c r="A79" t="s">
         <v>76</v>
       </c>
@@ -2269,7 +2277,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5">
       <c r="A80" t="s">
         <v>76</v>
       </c>
@@ -2286,7 +2294,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5">
       <c r="A81" t="s">
         <v>76</v>
       </c>
@@ -2303,7 +2311,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5">
       <c r="A82" t="s">
         <v>76</v>
       </c>
@@ -2320,7 +2328,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5">
       <c r="A83" t="s">
         <v>76</v>
       </c>
@@ -2337,7 +2345,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5">
       <c r="A84" t="s">
         <v>76</v>
       </c>
@@ -2354,7 +2362,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5">
       <c r="A85" t="s">
         <v>76</v>
       </c>
@@ -2371,7 +2379,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5">
       <c r="A86" t="s">
         <v>76</v>
       </c>
@@ -2388,7 +2396,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5">
       <c r="A87" t="s">
         <v>76</v>
       </c>
@@ -2405,7 +2413,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5">
       <c r="A88" t="s">
         <v>79</v>
       </c>
@@ -2422,7 +2430,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5">
       <c r="A89" t="s">
         <v>79</v>
       </c>
@@ -2439,7 +2447,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5">
       <c r="A90" t="s">
         <v>79</v>
       </c>
@@ -2456,7 +2464,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5">
       <c r="A91" t="s">
         <v>79</v>
       </c>
@@ -2473,7 +2481,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5">
       <c r="A92" t="s">
         <v>79</v>
       </c>
@@ -2490,7 +2498,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5">
       <c r="A93" t="s">
         <v>81</v>
       </c>
@@ -2507,7 +2515,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5">
       <c r="A94" t="s">
         <v>81</v>
       </c>
@@ -2524,7 +2532,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5">
       <c r="A95" t="s">
         <v>81</v>
       </c>
@@ -2541,7 +2549,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5">
       <c r="A96" t="s">
         <v>81</v>
       </c>
@@ -2558,7 +2566,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5">
       <c r="A97" t="s">
         <v>81</v>
       </c>
@@ -2575,7 +2583,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5">
       <c r="A98" t="s">
         <v>81</v>
       </c>
@@ -2592,7 +2600,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5">
       <c r="A99" t="s">
         <v>89</v>
       </c>
@@ -2609,7 +2617,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5">
       <c r="A100" t="s">
         <v>89</v>
       </c>
@@ -2626,7 +2634,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5">
       <c r="A101" t="s">
         <v>89</v>
       </c>
@@ -2643,7 +2651,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5">
       <c r="A102" t="s">
         <v>89</v>
       </c>
@@ -2660,7 +2668,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5">
       <c r="A103" t="s">
         <v>89</v>
       </c>
@@ -2677,7 +2685,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5">
       <c r="A104" t="s">
         <v>94</v>
       </c>
@@ -2694,7 +2702,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5">
       <c r="A105" t="s">
         <v>94</v>
       </c>
@@ -2711,7 +2719,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5">
       <c r="A106" t="s">
         <v>94</v>
       </c>
@@ -2728,7 +2736,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5">
       <c r="A107" t="s">
         <v>94</v>
       </c>
@@ -2745,7 +2753,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5">
       <c r="A108" t="s">
         <v>94</v>
       </c>
@@ -2762,7 +2770,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5">
       <c r="A109" t="s">
         <v>94</v>
       </c>
@@ -2779,7 +2787,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5">
       <c r="A110" t="s">
         <v>97</v>
       </c>
@@ -2796,7 +2804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5">
       <c r="A111" t="s">
         <v>97</v>
       </c>
@@ -2813,7 +2821,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5">
       <c r="A112" t="s">
         <v>97</v>
       </c>
@@ -2830,7 +2838,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5">
       <c r="A113" t="s">
         <v>97</v>
       </c>
@@ -2847,7 +2855,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5">
       <c r="A114" t="s">
         <v>97</v>
       </c>
@@ -2864,7 +2872,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5">
       <c r="A115" t="s">
         <v>99</v>
       </c>
@@ -2881,7 +2889,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5">
       <c r="A116" t="s">
         <v>99</v>
       </c>
@@ -2898,7 +2906,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5">
       <c r="A117" t="s">
         <v>99</v>
       </c>
@@ -2915,7 +2923,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5">
       <c r="A118" t="s">
         <v>99</v>
       </c>
@@ -2932,7 +2940,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5">
       <c r="A119" t="s">
         <v>99</v>
       </c>
@@ -2949,7 +2957,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5">
       <c r="A120" t="s">
         <v>99</v>
       </c>
@@ -2966,7 +2974,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5">
       <c r="A121" t="s">
         <v>99</v>
       </c>
@@ -2983,7 +2991,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5">
       <c r="A122" t="s">
         <v>101</v>
       </c>
@@ -3000,7 +3008,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5">
       <c r="A123" t="s">
         <v>101</v>
       </c>
@@ -3017,7 +3025,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5">
       <c r="A124" t="s">
         <v>101</v>
       </c>
@@ -3034,7 +3042,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5">
       <c r="A125" t="s">
         <v>101</v>
       </c>
@@ -3051,7 +3059,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5">
       <c r="A126" t="s">
         <v>101</v>
       </c>
@@ -3068,7 +3076,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5">
       <c r="A127" t="s">
         <v>101</v>
       </c>
@@ -3085,7 +3093,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5">
       <c r="A128" t="s">
         <v>103</v>
       </c>
@@ -3102,7 +3110,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5">
       <c r="A129" t="s">
         <v>103</v>
       </c>
@@ -3119,7 +3127,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5">
       <c r="A130" t="s">
         <v>103</v>
       </c>
@@ -3136,7 +3144,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5">
       <c r="A131" t="s">
         <v>103</v>
       </c>
@@ -3153,7 +3161,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5">
       <c r="A132" t="s">
         <v>103</v>
       </c>
@@ -3170,7 +3178,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5">
       <c r="A133" t="s">
         <v>103</v>
       </c>
@@ -3187,7 +3195,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5">
       <c r="A134" t="s">
         <v>103</v>
       </c>
@@ -3204,7 +3212,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5">
       <c r="A135" t="s">
         <v>103</v>
       </c>
@@ -3221,7 +3229,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5">
       <c r="A136" t="s">
         <v>103</v>
       </c>
@@ -3238,7 +3246,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5">
       <c r="A137" t="s">
         <v>112</v>
       </c>
@@ -3255,7 +3263,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5">
       <c r="A138" t="s">
         <v>112</v>
       </c>
@@ -3272,7 +3280,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5">
       <c r="A139" t="s">
         <v>112</v>
       </c>
@@ -3289,7 +3297,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5">
       <c r="A140" t="s">
         <v>112</v>
       </c>
@@ -3306,7 +3314,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5">
       <c r="A141" t="s">
         <v>112</v>
       </c>
@@ -3323,7 +3331,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5">
       <c r="A142" t="s">
         <v>112</v>
       </c>
@@ -3340,7 +3348,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5">
       <c r="A143" t="s">
         <v>112</v>
       </c>
@@ -3357,7 +3365,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5">
       <c r="A144" t="s">
         <v>118</v>
       </c>
@@ -3374,7 +3382,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5">
       <c r="A145" t="s">
         <v>118</v>
       </c>
@@ -3391,7 +3399,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5">
       <c r="A146" t="s">
         <v>118</v>
       </c>
@@ -3402,13 +3410,13 @@
         <v>7</v>
       </c>
       <c r="D146" t="s">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="E146" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5">
       <c r="A147" t="s">
         <v>118</v>
       </c>
@@ -3425,7 +3433,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5">
       <c r="A148" t="s">
         <v>118</v>
       </c>
@@ -3442,7 +3450,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5">
       <c r="A149" t="s">
         <v>118</v>
       </c>
@@ -3459,7 +3467,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5">
       <c r="A150" t="s">
         <v>118</v>
       </c>
@@ -3476,7 +3484,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5">
       <c r="A151" t="s">
         <v>118</v>
       </c>
@@ -3493,7 +3501,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5">
       <c r="A152" t="s">
         <v>118</v>
       </c>
@@ -3510,7 +3518,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5">
       <c r="A153" t="s">
         <v>127</v>
       </c>
@@ -3527,7 +3535,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5">
       <c r="A154" t="s">
         <v>127</v>
       </c>
@@ -3544,7 +3552,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5">
       <c r="A155" t="s">
         <v>127</v>
       </c>
@@ -3561,7 +3569,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5">
       <c r="A156" t="s">
         <v>127</v>
       </c>
@@ -3578,7 +3586,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5">
       <c r="A157" t="s">
         <v>127</v>
       </c>
@@ -3595,7 +3603,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5">
       <c r="A158" t="s">
         <v>127</v>
       </c>
@@ -3612,7 +3620,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5">
       <c r="A159" t="s">
         <v>127</v>
       </c>
@@ -3629,7 +3637,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5">
       <c r="A160" t="s">
         <v>132</v>
       </c>
@@ -3646,7 +3654,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5">
       <c r="A161" t="s">
         <v>132</v>
       </c>
@@ -3663,7 +3671,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5">
       <c r="A162" t="s">
         <v>132</v>
       </c>
@@ -3680,7 +3688,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5">
       <c r="A163" t="s">
         <v>132</v>
       </c>
@@ -3697,7 +3705,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5">
       <c r="A164" t="s">
         <v>132</v>
       </c>
@@ -3714,7 +3722,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5">
       <c r="A165" t="s">
         <v>132</v>
       </c>
@@ -3731,7 +3739,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5">
       <c r="A166" t="s">
         <v>132</v>
       </c>
@@ -3748,7 +3756,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5">
       <c r="A167" t="s">
         <v>132</v>
       </c>
@@ -3765,7 +3773,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5">
       <c r="A168" t="s">
         <v>140</v>
       </c>
@@ -3782,7 +3790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5">
       <c r="A169" t="s">
         <v>140</v>
       </c>
@@ -3799,7 +3807,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5">
       <c r="A170" t="s">
         <v>140</v>
       </c>
@@ -3816,7 +3824,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5">
       <c r="A171" t="s">
         <v>140</v>
       </c>
@@ -3833,7 +3841,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5">
       <c r="A172" t="s">
         <v>140</v>
       </c>
@@ -3850,7 +3858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5">
       <c r="A173" t="s">
         <v>140</v>
       </c>
@@ -3867,7 +3875,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5">
       <c r="A174" t="s">
         <v>140</v>
       </c>
@@ -3884,7 +3892,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5">
       <c r="A175" t="s">
         <v>140</v>
       </c>
@@ -3901,7 +3909,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5">
       <c r="A176" t="s">
         <v>148</v>
       </c>
@@ -3918,7 +3926,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5">
       <c r="A177" t="s">
         <v>148</v>
       </c>
@@ -3935,7 +3943,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5">
       <c r="A178" t="s">
         <v>148</v>
       </c>
@@ -3952,7 +3960,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5">
       <c r="A179" t="s">
         <v>148</v>
       </c>
@@ -3969,7 +3977,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5">
       <c r="A180" t="s">
         <v>148</v>
       </c>
@@ -3986,7 +3994,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5">
       <c r="A181" t="s">
         <v>148</v>
       </c>
@@ -4003,7 +4011,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5">
       <c r="A182" t="s">
         <v>152</v>
       </c>
@@ -4020,7 +4028,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5">
       <c r="A183" t="s">
         <v>152</v>
       </c>
@@ -4037,7 +4045,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5">
       <c r="A184" t="s">
         <v>152</v>
       </c>
@@ -4054,7 +4062,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5">
       <c r="A185" t="s">
         <v>152</v>
       </c>
@@ -4071,7 +4079,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5">
       <c r="A186" t="s">
         <v>152</v>
       </c>
@@ -4088,7 +4096,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5">
       <c r="A187" t="s">
         <v>152</v>
       </c>
@@ -4105,7 +4113,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5">
       <c r="A188" t="s">
         <v>152</v>
       </c>
@@ -4122,7 +4130,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5">
       <c r="A189" t="s">
         <v>152</v>
       </c>
@@ -4139,7 +4147,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5">
       <c r="A190" t="s">
         <v>161</v>
       </c>
@@ -4156,7 +4164,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5">
       <c r="A191" t="s">
         <v>161</v>
       </c>
@@ -4173,7 +4181,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5">
       <c r="A192" t="s">
         <v>161</v>
       </c>
@@ -4190,7 +4198,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5">
       <c r="A193" t="s">
         <v>161</v>
       </c>
@@ -4207,7 +4215,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5">
       <c r="A194" t="s">
         <v>161</v>
       </c>
@@ -4224,7 +4232,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5">
       <c r="A195" t="s">
         <v>161</v>
       </c>
@@ -4241,7 +4249,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5">
       <c r="A196" t="s">
         <v>161</v>
       </c>
@@ -4258,7 +4266,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5">
       <c r="A197" t="s">
         <v>161</v>
       </c>
@@ -4275,7 +4283,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5">
       <c r="A198" t="s">
         <v>166</v>
       </c>
@@ -4292,7 +4300,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5">
       <c r="A199" t="s">
         <v>166</v>
       </c>
@@ -4309,7 +4317,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5">
       <c r="A200" t="s">
         <v>166</v>
       </c>
@@ -4326,7 +4334,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5">
       <c r="A201" t="s">
         <v>166</v>
       </c>
@@ -4343,7 +4351,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5">
       <c r="A202" t="s">
         <v>166</v>
       </c>
@@ -4360,7 +4368,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5">
       <c r="A203" t="s">
         <v>168</v>
       </c>
@@ -4377,7 +4385,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5">
       <c r="A204" t="s">
         <v>168</v>
       </c>
@@ -4394,7 +4402,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5">
       <c r="A205" t="s">
         <v>168</v>
       </c>
@@ -4411,7 +4419,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5">
       <c r="A206" t="s">
         <v>168</v>
       </c>
@@ -4428,7 +4436,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5">
       <c r="A207" t="s">
         <v>168</v>
       </c>
@@ -4445,7 +4453,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5">
       <c r="A208" t="s">
         <v>168</v>
       </c>
@@ -4462,7 +4470,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5">
       <c r="A209" t="s">
         <v>168</v>
       </c>
@@ -4479,7 +4487,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5">
       <c r="A210" t="s">
         <v>168</v>
       </c>
@@ -4496,7 +4504,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5">
       <c r="A211" t="s">
         <v>171</v>
       </c>
@@ -4513,7 +4521,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5">
       <c r="A212" t="s">
         <v>171</v>
       </c>
@@ -4530,7 +4538,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5">
       <c r="A213" t="s">
         <v>171</v>
       </c>
@@ -4547,7 +4555,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5">
       <c r="A214" t="s">
         <v>171</v>
       </c>
@@ -4564,7 +4572,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5">
       <c r="A215" t="s">
         <v>171</v>
       </c>
@@ -4581,7 +4589,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5">
       <c r="A216" t="s">
         <v>171</v>
       </c>
@@ -4598,7 +4606,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5">
       <c r="A217" t="s">
         <v>171</v>
       </c>
@@ -4615,7 +4623,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5">
       <c r="A218" t="s">
         <v>171</v>
       </c>
@@ -4632,7 +4640,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5">
       <c r="A219" t="s">
         <v>171</v>
       </c>
@@ -4651,6 +4659,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>